<commit_message>
feat: decouple programs from schedule
</commit_message>
<xml_diff>
--- a/Aulas_Con_Formulas_Fernando.xlsx
+++ b/Aulas_Con_Formulas_Fernando.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -595,11 +595,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>4to</t>
-        </is>
-      </c>
+      <c r="A6" t="inlineStr"/>
       <c r="C6">
         <f>SUSTITUIR(ESPACIOS(CONCATENAR(SI(C111!$C$5=C$2;C111!$B$1 &amp; " "; "")SI(C121!$C$5=C$2;C121!$B$1 &amp; " "; "")SI(C122!$C$5=C$2;C122!$B$1 &amp; " "; "")SI(C211!$C$5=C$2;C211!$B$1 &amp; " "; "")SI(C212!$C$5=C$2;C212!$B$1 &amp; " "; "")SI(C311!$C$5=C$2;C311!$B$1 &amp; " "; "")SI(C312!$C$5=C$2;C312!$B$1 &amp; " "; "")SI(C411!$C$5=C$2;C411!$B$1 &amp; " "; "")SI(C412!$C$5=C$2;C412!$B$1 &amp; " "; "")SI(D111!$C$5=C$2;D111!$B$1 &amp; " "; "")SI(D211!$C$5=C$2;D211!$B$1 &amp; " "; "")SI(D311!$C$5=C$2;D311!$B$1 &amp; " "; "")SI(D411!$C$5=C$2;D411!$B$1 &amp; " "; "")SI(M111!$C$5=C$2;M111!$B$1 &amp; " "; "")SI(M211!$C$5=C$2;M211!$B$1 &amp; " "; "")SI(M311!$C$5=C$2;M311!$B$1 &amp; " "; "")SI(M411!$C$5=C$2;M411!$B$1 &amp; " "; ""))); " "; ",")</f>
         <v/>
@@ -644,7 +640,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>5to</t>
+          <t>4to</t>
         </is>
       </c>
       <c r="C7">
@@ -691,7 +687,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>6to</t>
+          <t>5to</t>
         </is>
       </c>
       <c r="C8">
@@ -738,7 +734,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Martes</t>
+          <t>6to</t>
         </is>
       </c>
       <c r="C9">
@@ -785,7 +781,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1ro</t>
+          <t>Martes</t>
         </is>
       </c>
       <c r="C10">
@@ -832,7 +828,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2do</t>
+          <t>1ro</t>
         </is>
       </c>
       <c r="C11">
@@ -879,7 +875,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>3ro</t>
+          <t>2do</t>
         </is>
       </c>
       <c r="C12">
@@ -926,7 +922,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>4to</t>
+          <t>3ro</t>
         </is>
       </c>
       <c r="C13">
@@ -971,11 +967,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>5to</t>
-        </is>
-      </c>
+      <c r="A14" t="inlineStr"/>
       <c r="C14">
         <f>SUSTITUIR(ESPACIOS(CONCATENAR(SI(C111!$C$5=C$2;C111!$B$1 &amp; " "; "")SI(C121!$C$5=C$2;C121!$B$1 &amp; " "; "")SI(C122!$C$5=C$2;C122!$B$1 &amp; " "; "")SI(C211!$C$5=C$2;C211!$B$1 &amp; " "; "")SI(C212!$C$5=C$2;C212!$B$1 &amp; " "; "")SI(C311!$C$5=C$2;C311!$B$1 &amp; " "; "")SI(C312!$C$5=C$2;C312!$B$1 &amp; " "; "")SI(C411!$C$5=C$2;C411!$B$1 &amp; " "; "")SI(C412!$C$5=C$2;C412!$B$1 &amp; " "; "")SI(D111!$C$5=C$2;D111!$B$1 &amp; " "; "")SI(D211!$C$5=C$2;D211!$B$1 &amp; " "; "")SI(D311!$C$5=C$2;D311!$B$1 &amp; " "; "")SI(D411!$C$5=C$2;D411!$B$1 &amp; " "; "")SI(M111!$C$5=C$2;M111!$B$1 &amp; " "; "")SI(M211!$C$5=C$2;M211!$B$1 &amp; " "; "")SI(M311!$C$5=C$2;M311!$B$1 &amp; " "; "")SI(M411!$C$5=C$2;M411!$B$1 &amp; " "; ""))); " "; ",")</f>
         <v/>
@@ -1020,7 +1012,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>6to</t>
+          <t>4to</t>
         </is>
       </c>
       <c r="C15">
@@ -1067,7 +1059,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Miércoles</t>
+          <t>5to</t>
         </is>
       </c>
       <c r="C16">
@@ -1114,7 +1106,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1ro</t>
+          <t>6to</t>
         </is>
       </c>
       <c r="C17">
@@ -1161,131 +1153,154 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2do</t>
+          <t>Miércoles</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>3ro</t>
+          <t>1ro</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>4to</t>
+          <t>2do</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>5to</t>
+          <t>3ro</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>6to</t>
-        </is>
-      </c>
+      <c r="A22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Jueves</t>
+          <t>4to</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1ro</t>
+          <t>5to</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2do</t>
+          <t>6to</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>3ro</t>
+          <t>Jueves</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>4to</t>
+          <t>1ro</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>5to</t>
+          <t>2do</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>6to</t>
+          <t>3ro</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Viernes</t>
-        </is>
-      </c>
+      <c r="A30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1ro</t>
+          <t>4to</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2do</t>
+          <t>5to</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>3ro</t>
+          <t>6to</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>4to</t>
+          <t>Viernes</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>5to</t>
+          <t>1ro</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
+        <is>
+          <t>2do</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>3ro</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>4to</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>5to</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
         <is>
           <t>6to</t>
         </is>

</xml_diff>